<commit_message>
finalized stucture and moved data to excel sheet
</commit_message>
<xml_diff>
--- a/MarketingMail/templates/excel(marketingmail).xlsx
+++ b/MarketingMail/templates/excel(marketingmail).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UTHIHI\PycharmProjects\MoamProject\MarketingMail\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{696FAAE4-413E-4265-A52F-402A29AC5F0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A92CCD5-3E69-4A2E-802C-45E7FB447691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EE254522-B9A6-4ECE-95C9-945019AE9520}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EE254522-B9A6-4ECE-95C9-945019AE9520}"/>
   </bookViews>
   <sheets>
     <sheet name="Maatwerk Notes nieuw" sheetId="2" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="12">
   <si>
     <t>BNP Paribas Issuance B.V. (Moody's: Aa3 / Fitch: AA- / S&amp;P: A+)</t>
   </si>
@@ -129,9 +129,6 @@
   </si>
   <si>
     <t>BNP Paribas Issuance B.V. (Moody's: A1 / Fitch: A+ / S&amp;P: A+)</t>
-  </si>
-  <si>
-    <t>dw</t>
   </si>
 </sst>
 </file>
@@ -286,7 +283,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -298,22 +295,20 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="10" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -322,13 +317,11 @@
     <xf numFmtId="49" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="10" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -492,148 +485,47 @@
           <cell r="D4" t="str">
             <v>Index Garantie Note</v>
           </cell>
-          <cell r="F4" t="str">
-            <v>Product:</v>
-          </cell>
-          <cell r="G4" t="str">
-            <v>Memory Coupon</v>
-          </cell>
-          <cell r="J4" t="str">
-            <v>Memory Coupon</v>
-          </cell>
           <cell r="L4" t="str">
             <v>Product:</v>
           </cell>
-          <cell r="M4" t="str">
-            <v>Memory Coupon</v>
-          </cell>
         </row>
         <row r="5">
-          <cell r="D5">
-            <v>5</v>
-          </cell>
-          <cell r="F5" t="str">
-            <v>T+x</v>
-          </cell>
-          <cell r="G5">
-            <v>5</v>
-          </cell>
-          <cell r="J5">
-            <v>5</v>
-          </cell>
           <cell r="L5" t="str">
             <v>T+x</v>
-          </cell>
-          <cell r="M5">
-            <v>5</v>
           </cell>
         </row>
         <row r="6">
           <cell r="D6" t="str">
             <v>5Y</v>
           </cell>
-          <cell r="F6" t="str">
-            <v>Maturity:</v>
-          </cell>
-          <cell r="G6" t="str">
-            <v>5Y</v>
-          </cell>
-          <cell r="J6" t="str">
-            <v>7Y</v>
-          </cell>
           <cell r="L6" t="str">
             <v>Maturity:</v>
-          </cell>
-          <cell r="M6" t="str">
-            <v>7Y</v>
           </cell>
         </row>
         <row r="7">
           <cell r="D7" t="str">
             <v>SX5E</v>
           </cell>
-          <cell r="F7" t="str">
-            <v>OW:</v>
-          </cell>
-          <cell r="G7" t="str">
-            <v>SX5E</v>
-          </cell>
-          <cell r="J7" t="str">
-            <v>SX5E</v>
-          </cell>
           <cell r="L7" t="str">
             <v>OW:</v>
           </cell>
-          <cell r="M7" t="str">
-            <v>SX5E</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="J9" t="str">
-            <v>SPX</v>
-          </cell>
-          <cell r="M9" t="str">
-            <v>SPX</v>
-          </cell>
         </row>
         <row r="11">
-          <cell r="D11" t="str">
-            <v>EUR</v>
-          </cell>
-          <cell r="F11" t="str">
-            <v>Currency:</v>
-          </cell>
-          <cell r="G11" t="str">
-            <v>EUR</v>
-          </cell>
-          <cell r="J11" t="str">
-            <v>EUR</v>
-          </cell>
           <cell r="L11" t="str">
             <v>Currency:</v>
-          </cell>
-          <cell r="M11" t="str">
-            <v>EUR</v>
           </cell>
         </row>
         <row r="13">
           <cell r="D13" t="str">
             <v>VLK</v>
           </cell>
-          <cell r="F13" t="str">
-            <v>Issuer:</v>
-          </cell>
-          <cell r="G13" t="str">
-            <v>VLK</v>
-          </cell>
-          <cell r="J13" t="str">
-            <v>VLK</v>
-          </cell>
           <cell r="L13" t="str">
             <v>Issuer:</v>
           </cell>
-          <cell r="M13" t="str">
-            <v>BNP</v>
-          </cell>
         </row>
         <row r="16">
-          <cell r="D16" t="str">
-            <v>50k</v>
-          </cell>
-          <cell r="F16" t="str">
-            <v>Denomination:</v>
-          </cell>
-          <cell r="G16" t="str">
-            <v>100k</v>
-          </cell>
-          <cell r="J16" t="str">
-            <v>100k</v>
-          </cell>
           <cell r="L16" t="str">
             <v>Denomination:</v>
-          </cell>
-          <cell r="M16" t="str">
-            <v>100k</v>
           </cell>
         </row>
         <row r="18">
@@ -643,17 +535,11 @@
           <cell r="F18" t="str">
             <v>Premie:</v>
           </cell>
-          <cell r="G18">
-            <v>7</v>
-          </cell>
           <cell r="I18" t="str">
             <v>Premie:</v>
           </cell>
           <cell r="L18" t="str">
             <v>Premie:</v>
-          </cell>
-          <cell r="M18">
-            <v>5.2</v>
           </cell>
         </row>
         <row r="19">
@@ -663,9 +549,6 @@
           <cell r="F19" t="str">
             <v>Aflossingsbarriere:</v>
           </cell>
-          <cell r="G19" t="str">
-            <v>nvt</v>
-          </cell>
           <cell r="I19" t="str">
             <v>Aflossingsbarriere:</v>
           </cell>
@@ -680,9 +563,6 @@
           <cell r="F20" t="str">
             <v>Couponbarriere:</v>
           </cell>
-          <cell r="G20">
-            <v>90</v>
-          </cell>
           <cell r="I20" t="str">
             <v>Couponbarriere:</v>
           </cell>
@@ -697,9 +577,6 @@
           <cell r="F21" t="str">
             <v>Bescherming:</v>
           </cell>
-          <cell r="G21">
-            <v>70</v>
-          </cell>
           <cell r="I21" t="str">
             <v>Bescherming:</v>
           </cell>
@@ -708,34 +585,11 @@
           </cell>
         </row>
         <row r="25">
-          <cell r="D25">
-            <v>0</v>
-          </cell>
-          <cell r="F25" t="str">
-            <v>Fixing if not today +</v>
-          </cell>
-          <cell r="G25">
-            <v>0</v>
-          </cell>
-          <cell r="J25">
-            <v>0</v>
-          </cell>
           <cell r="L25" t="str">
             <v>Fixing if not today +</v>
           </cell>
-          <cell r="M25">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="159">
-          <cell r="F159" t="str">
-            <v>denom</v>
-          </cell>
         </row>
         <row r="165">
-          <cell r="F165" t="str">
-            <v>Look Ups</v>
-          </cell>
           <cell r="K165" t="str">
             <v>OW:</v>
           </cell>
@@ -755,12 +609,6 @@
           </cell>
         </row>
         <row r="167">
-          <cell r="F167" t="str">
-            <v>VLK</v>
-          </cell>
-          <cell r="G167" t="str">
-            <v>Van Lanschot Kempen N.V. (Fitch: A- / S&amp;P: BBB+)</v>
-          </cell>
           <cell r="K167" t="str">
             <v>SX5E</v>
           </cell>
@@ -775,12 +623,6 @@
           </cell>
         </row>
         <row r="168">
-          <cell r="F168" t="str">
-            <v>BNP</v>
-          </cell>
-          <cell r="G168" t="str">
-            <v>BNP Paribas Issuance B.V. (Moody's: Aa3 / Fitch: AA- / S&amp;P: A+)</v>
-          </cell>
           <cell r="K168" t="str">
             <v>SX7E</v>
           </cell>
@@ -795,12 +637,6 @@
           </cell>
         </row>
         <row r="169">
-          <cell r="F169" t="str">
-            <v>ING</v>
-          </cell>
-          <cell r="G169" t="str">
-            <v>ING Bank N.V. (Fitch: A / S&amp;P: A)</v>
-          </cell>
           <cell r="K169" t="str">
             <v>SD3E</v>
           </cell>
@@ -1408,14 +1244,14 @@
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
-      <c r="R10" s="11" t="s">
+      <c r="R10" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="S10" s="11"/>
-      <c r="T10" s="11"/>
-      <c r="U10" s="11"/>
-      <c r="V10" s="11"/>
-      <c r="W10" s="11"/>
+      <c r="S10" s="19"/>
+      <c r="T10" s="19"/>
+      <c r="U10" s="19"/>
+      <c r="V10" s="19"/>
+      <c r="W10" s="19"/>
     </row>
     <row r="11" spans="1:23" ht="157.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
@@ -1434,114 +1270,114 @@
     </row>
     <row r="12" spans="1:23" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
-      <c r="B12" s="12" t="str">
+      <c r="B12" s="20" t="str">
         <f>"Van Lanschot Kempen heeft de volgende maatwerk producten gelanceerd. Vanaf heden kan zolang er Notes beschikbaar zijn vanaf "&amp;
 '[2]Marketing MAIL'!D171 &amp;
 " mee gedaan worden in deze producten tegen de actuele laatprijs. Neem voor de actuele laatprijs en/of het opgeven van een order contact op met Van Lanschot Kempen Structured Products. "&amp;
 "Hieronder vindt u beknopt de belangrijkste kenmerken van de nieuwe maatwerk producten. De volledige documentatie verschijnt binnenkort op www.markets.vanlanschotkempen.com."</f>
         <v>Van Lanschot Kempen heeft de volgende maatwerk producten gelanceerd. Vanaf heden kan zolang er Notes beschikbaar zijn vanaf EUR 50k mee gedaan worden in deze producten tegen de actuele laatprijs. Neem voor de actuele laatprijs en/of het opgeven van een order contact op met Van Lanschot Kempen Structured Products. Hieronder vindt u beknopt de belangrijkste kenmerken van de nieuwe maatwerk producten. De volledige documentatie verschijnt binnenkort op www.markets.vanlanschotkempen.com.</v>
       </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="12"/>
-      <c r="L12" s="12"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="20"/>
+      <c r="L12" s="20"/>
       <c r="M12" s="1"/>
-      <c r="R12" s="11" t="s">
+      <c r="R12" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="S12" s="11"/>
-      <c r="T12" s="11"/>
-      <c r="U12" s="11"/>
-      <c r="V12" s="11"/>
-      <c r="W12" s="11"/>
+      <c r="S12" s="19"/>
+      <c r="T12" s="19"/>
+      <c r="U12" s="19"/>
+      <c r="V12" s="19"/>
+      <c r="W12" s="19"/>
     </row>
     <row r="13" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12"/>
-      <c r="L13" s="12"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
+      <c r="J13" s="20"/>
+      <c r="K13" s="20"/>
+      <c r="L13" s="20"/>
       <c r="M13" s="1"/>
     </row>
     <row r="14" spans="1:23" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="12"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
+      <c r="I14" s="20"/>
+      <c r="J14" s="20"/>
+      <c r="K14" s="20"/>
+      <c r="L14" s="20"/>
       <c r="M14" s="1"/>
-      <c r="R14" s="11" t="s">
+      <c r="R14" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="S14" s="11"/>
-      <c r="T14" s="11"/>
-      <c r="U14" s="11"/>
-      <c r="V14" s="11"/>
-      <c r="W14" s="11"/>
+      <c r="S14" s="19"/>
+      <c r="T14" s="19"/>
+      <c r="U14" s="19"/>
+      <c r="V14" s="19"/>
+      <c r="W14" s="19"/>
     </row>
     <row r="15" spans="1:23" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="12"/>
-      <c r="L15" s="12"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="20"/>
+      <c r="L15" s="20"/>
       <c r="M15" s="1"/>
     </row>
     <row r="16" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="12"/>
-      <c r="J16" s="12"/>
-      <c r="K16" s="12"/>
-      <c r="L16" s="12"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="20"/>
+      <c r="L16" s="20"/>
       <c r="M16" s="1"/>
     </row>
     <row r="17" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="12"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="12"/>
-      <c r="L17" s="12"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="20"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="20"/>
+      <c r="L17" s="20"/>
       <c r="M17" s="1"/>
       <c r="S17" s="2" t="str">
         <f>'[2]Marketing MAIL'!D13 &amp; " " &amp; '[2]Marketing MAIL'!D4 &amp; " " &amp;
@@ -1584,14 +1420,7 @@
     </row>
     <row r="20" spans="1:25" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1"/>
-      <c r="B20" s="4" t="str">
-        <f>'[2]Marketing MAIL'!D13 &amp; " " &amp; '[2]Marketing MAIL'!D4 &amp; " " &amp;
-VLOOKUP('[2]Marketing MAIL'!D7,'[2]Marketing MAIL'!P:Q,2,FALSE)&amp;
-IF('[2]Marketing MAIL'!D9="",""," " &amp; VLOOKUP('[2]Marketing MAIL'!D8,'[2]Marketing MAIL'!P:Q,2,FALSE))&amp;
-" " &amp;
-"26-" &amp;(26+VALUE(LEFT('[2]Marketing MAIL'!D6,LEN('[2]Marketing MAIL'!D6)-1)))</f>
-        <v>VLK Index Garantie Note Eurozone 26-31</v>
-      </c>
+      <c r="B20" s="4"/>
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
       <c r="E20" s="5"/>
@@ -1621,22 +1450,19 @@
     </row>
     <row r="22" spans="1:25" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1"/>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
-      <c r="G22" s="14" t="str">
-        <f>_xlfn.XLOOKUP('[2]Marketing MAIL'!D13,'[2]Marketing MAIL'!F:F,'[2]Marketing MAIL'!G:G)</f>
-        <v>Van Lanschot Kempen N.V. (Fitch: A- / S&amp;P: BBB+)</v>
-      </c>
-      <c r="H22" s="14"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="14"/>
-      <c r="K22" s="14"/>
-      <c r="L22" s="14"/>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13"/>
+      <c r="I22" s="13"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13"/>
+      <c r="L22" s="13"/>
       <c r="M22" s="1"/>
       <c r="Q22" s="2" t="s">
         <v>4</v>
@@ -1663,22 +1489,19 @@
     </row>
     <row r="24" spans="1:25" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1"/>
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
-      <c r="G24" s="14" t="str">
-        <f ca="1">"TBD/TBD/" &amp; TEXT(WORKDAY(TODAY(),'[2]Marketing MAIL'!D5+'[2]Marketing MAIL'!D25 +2),"d mmm yyyy")</f>
-        <v>TBD/TBD/28 Apr 2026</v>
-      </c>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
+      <c r="G24" s="13"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="13"/>
+      <c r="J24" s="13"/>
+      <c r="K24" s="13"/>
+      <c r="L24" s="13"/>
       <c r="M24" s="1"/>
     </row>
     <row r="25" spans="1:25" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1698,22 +1521,19 @@
     </row>
     <row r="26" spans="1:25" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
-      <c r="G26" s="14" t="str">
-        <f>'[2]Marketing MAIL'!D11 &amp; " " &amp; TEXT(_xlfn.NUMBERVALUE(SUBSTITUTE(LOWER(TRIM('[2]Marketing MAIL'!D16)),"k",""), ",", ".")*1000, "#,##0")</f>
-        <v>EUR 50,000</v>
-      </c>
-      <c r="H26" s="14"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="14"/>
-      <c r="K26" s="14"/>
-      <c r="L26" s="14"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13"/>
+      <c r="I26" s="13"/>
+      <c r="J26" s="13"/>
+      <c r="K26" s="13"/>
+      <c r="L26" s="13"/>
       <c r="M26" s="1"/>
     </row>
     <row r="27" spans="1:25" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1733,22 +1553,19 @@
     </row>
     <row r="28" spans="1:25" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
-      <c r="B28" s="13" t="s">
+      <c r="B28" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
-      <c r="G28" s="14" t="str">
-        <f>SUBSTITUTE('[2]Marketing MAIL'!D6,"Y"," jaar")</f>
-        <v>5 jaar</v>
-      </c>
-      <c r="H28" s="14"/>
-      <c r="I28" s="14"/>
-      <c r="J28" s="14"/>
-      <c r="K28" s="14"/>
-      <c r="L28" s="14"/>
+      <c r="G28" s="13"/>
+      <c r="H28" s="13"/>
+      <c r="I28" s="13"/>
+      <c r="J28" s="13"/>
+      <c r="K28" s="13"/>
+      <c r="L28" s="13"/>
       <c r="M28" s="1"/>
     </row>
     <row r="29" spans="1:25" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1768,32 +1585,26 @@
     </row>
     <row r="30" spans="1:25" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1"/>
-      <c r="B30" s="13" t="s">
+      <c r="B30" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
-      <c r="G30" s="15" t="str">
-        <f>_xlfn.TEXTJOIN("/",TRUE,_xlfn.XLOOKUP('[2]Marketing MAIL'!D7,'[2]Marketing MAIL'!K:K,'[2]Marketing MAIL'!L:L,""),_xlfn.XLOOKUP('[2]Marketing MAIL'!D8,'[2]Marketing MAIL'!K:K,'[2]Marketing MAIL'!L:L,""),_xlfn.XLOOKUP('[2]Marketing MAIL'!D9,'[2]Marketing MAIL'!K:K,'[2]Marketing MAIL'!L:L,""),"")</f>
-        <v>EURO STOXX 50 Index</v>
-      </c>
-      <c r="H30" s="15"/>
-      <c r="I30" s="15"/>
-      <c r="J30" s="15"/>
-      <c r="K30" s="17" t="str">
-        <f ca="1">"Startwaarde: TBD(" &amp; TEXT(WORKDAY(TODAY(),'[2]Marketing MAIL'!D25),"[$-nl-NL]d mmm yy")&amp; ")"</f>
-        <v>Startwaarde: TBD(17 apr 26)</v>
-      </c>
+      <c r="G30" s="16"/>
+      <c r="H30" s="16"/>
+      <c r="I30" s="16"/>
+      <c r="J30" s="16"/>
+      <c r="K30" s="17"/>
       <c r="L30" s="17"/>
       <c r="M30" s="1"/>
-      <c r="R30" s="15" t="s">
+      <c r="R30" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="S30" s="15"/>
-      <c r="T30" s="15"/>
-      <c r="U30" s="15"/>
+      <c r="S30" s="16"/>
+      <c r="T30" s="16"/>
+      <c r="U30" s="16"/>
       <c r="Y30" s="8">
         <f>2.103/4</f>
         <v>0.52575000000000005</v>
@@ -1816,20 +1627,20 @@
     </row>
     <row r="32" spans="1:25" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1"/>
-      <c r="B32" s="16" t="str">
+      <c r="B32" s="14" t="str">
         <f>'[2]Marketing MAIL'!C18</f>
         <v>Protection:</v>
       </c>
-      <c r="C32" s="16"/>
-      <c r="D32" s="16"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
-      <c r="G32" s="19"/>
-      <c r="H32" s="19"/>
-      <c r="I32" s="19"/>
-      <c r="J32" s="19"/>
-      <c r="K32" s="19"/>
-      <c r="L32" s="19"/>
+      <c r="G32" s="15"/>
+      <c r="H32" s="15"/>
+      <c r="I32" s="15"/>
+      <c r="J32" s="15"/>
+      <c r="K32" s="15"/>
+      <c r="L32" s="15"/>
       <c r="M32" s="1"/>
     </row>
     <row r="33" spans="1:19" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1849,20 +1660,20 @@
     </row>
     <row r="34" spans="1:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
-      <c r="B34" s="13" t="str">
+      <c r="B34" s="12" t="str">
         <f>'[2]Marketing MAIL'!C19</f>
         <v>Participatiegraad:</v>
       </c>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
+      <c r="C34" s="12"/>
+      <c r="D34" s="12"/>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
-      <c r="G34" s="19"/>
-      <c r="H34" s="19"/>
-      <c r="I34" s="19"/>
-      <c r="J34" s="19"/>
-      <c r="K34" s="19"/>
-      <c r="L34" s="19"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="15"/>
+      <c r="I34" s="15"/>
+      <c r="J34" s="15"/>
+      <c r="K34" s="15"/>
+      <c r="L34" s="15"/>
       <c r="M34" s="1"/>
       <c r="R34" s="18" t="s">
         <v>10</v>
@@ -1877,7 +1688,7 @@
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
       <c r="G35" s="7"/>
-      <c r="H35" s="20"/>
+      <c r="H35" s="11"/>
       <c r="I35" s="7"/>
       <c r="J35" s="7"/>
       <c r="K35" s="7"/>
@@ -1886,20 +1697,20 @@
     </row>
     <row r="36" spans="1:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1"/>
-      <c r="B36" s="13" t="str">
+      <c r="B36" s="12" t="str">
         <f>'[2]Marketing MAIL'!C20</f>
         <v>Max redemp:</v>
       </c>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
+      <c r="C36" s="12"/>
+      <c r="D36" s="12"/>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
-      <c r="G36" s="19"/>
-      <c r="H36" s="19"/>
-      <c r="I36" s="19"/>
-      <c r="J36" s="19"/>
-      <c r="K36" s="19"/>
-      <c r="L36" s="19"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="15"/>
+      <c r="I36" s="15"/>
+      <c r="J36" s="15"/>
+      <c r="K36" s="15"/>
+      <c r="L36" s="15"/>
       <c r="M36" s="1"/>
     </row>
     <row r="37" spans="1:19" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1919,20 +1730,20 @@
     </row>
     <row r="38" spans="1:19" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1"/>
-      <c r="B38" s="13" t="str">
+      <c r="B38" s="12" t="str">
         <f>'[2]Marketing MAIL'!C21</f>
         <v>Middeling:</v>
       </c>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
-      <c r="G38" s="19"/>
-      <c r="H38" s="19"/>
-      <c r="I38" s="19"/>
-      <c r="J38" s="19"/>
-      <c r="K38" s="19"/>
-      <c r="L38" s="19"/>
+      <c r="G38" s="15"/>
+      <c r="H38" s="15"/>
+      <c r="I38" s="15"/>
+      <c r="J38" s="15"/>
+      <c r="K38" s="15"/>
+      <c r="L38" s="15"/>
       <c r="M38" s="1"/>
       <c r="R38" s="2" t="s">
         <v>11</v>
@@ -1985,9 +1796,7 @@
     </row>
     <row r="42" spans="1:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1"/>
-      <c r="B42" s="4" t="s">
-        <v>12</v>
-      </c>
+      <c r="B42" s="4"/>
       <c r="C42" s="5"/>
       <c r="D42" s="5"/>
       <c r="E42" s="5"/>
@@ -2017,22 +1826,19 @@
     </row>
     <row r="44" spans="1:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1"/>
-      <c r="B44" s="13" t="s">
+      <c r="B44" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C44" s="13"/>
-      <c r="D44" s="13"/>
+      <c r="C44" s="12"/>
+      <c r="D44" s="12"/>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
-      <c r="G44" s="14" t="str">
-        <f>_xlfn.XLOOKUP('[2]Marketing MAIL'!G13,'[2]Marketing MAIL'!F:F,'[2]Marketing MAIL'!G:G)</f>
-        <v>Van Lanschot Kempen N.V. (Fitch: A- / S&amp;P: BBB+)</v>
-      </c>
-      <c r="H44" s="14"/>
-      <c r="I44" s="14"/>
-      <c r="J44" s="14"/>
-      <c r="K44" s="14"/>
-      <c r="L44" s="14"/>
+      <c r="G44" s="13"/>
+      <c r="H44" s="13"/>
+      <c r="I44" s="13"/>
+      <c r="J44" s="13"/>
+      <c r="K44" s="13"/>
+      <c r="L44" s="13"/>
       <c r="M44" s="1"/>
     </row>
     <row r="45" spans="1:19" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2052,22 +1858,19 @@
     </row>
     <row r="46" spans="1:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1"/>
-      <c r="B46" s="13" t="s">
+      <c r="B46" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C46" s="13"/>
-      <c r="D46" s="13"/>
+      <c r="C46" s="12"/>
+      <c r="D46" s="12"/>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
-      <c r="G46" s="14" t="str">
-        <f ca="1">"TBD/TBD/" &amp; TEXT(WORKDAY(TODAY(),'[2]Marketing MAIL'!G5+'[2]Marketing MAIL'!G25 +2),"d mmm yyyy")</f>
-        <v>TBD/TBD/28 Apr 2026</v>
-      </c>
-      <c r="H46" s="14"/>
-      <c r="I46" s="14"/>
-      <c r="J46" s="14"/>
-      <c r="K46" s="14"/>
-      <c r="L46" s="14"/>
+      <c r="G46" s="13"/>
+      <c r="H46" s="13"/>
+      <c r="I46" s="13"/>
+      <c r="J46" s="13"/>
+      <c r="K46" s="13"/>
+      <c r="L46" s="13"/>
       <c r="M46" s="1"/>
     </row>
     <row r="47" spans="1:19" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2087,22 +1890,19 @@
     </row>
     <row r="48" spans="1:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1"/>
-      <c r="B48" s="13" t="s">
+      <c r="B48" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
+      <c r="C48" s="12"/>
+      <c r="D48" s="12"/>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
-      <c r="G48" s="14" t="str">
-        <f>'[2]Marketing MAIL'!G11 &amp; " " &amp; TEXT(_xlfn.NUMBERVALUE(SUBSTITUTE(LOWER(TRIM('[2]Marketing MAIL'!G16)),"k",""), ",", ".")*1000, "#,##0")</f>
-        <v>EUR 100,000</v>
-      </c>
-      <c r="H48" s="14"/>
-      <c r="I48" s="14"/>
-      <c r="J48" s="14"/>
-      <c r="K48" s="14"/>
-      <c r="L48" s="14"/>
+      <c r="G48" s="13"/>
+      <c r="H48" s="13"/>
+      <c r="I48" s="13"/>
+      <c r="J48" s="13"/>
+      <c r="K48" s="13"/>
+      <c r="L48" s="13"/>
       <c r="M48" s="1"/>
     </row>
     <row r="49" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2122,22 +1922,19 @@
     </row>
     <row r="50" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1"/>
-      <c r="B50" s="13" t="s">
+      <c r="B50" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C50" s="13"/>
-      <c r="D50" s="13"/>
+      <c r="C50" s="12"/>
+      <c r="D50" s="12"/>
       <c r="E50" s="1"/>
       <c r="F50" s="1"/>
-      <c r="G50" s="14" t="str">
-        <f>SUBSTITUTE('[2]Marketing MAIL'!G6,"Y"," jaar")</f>
-        <v>5 jaar</v>
-      </c>
-      <c r="H50" s="14"/>
-      <c r="I50" s="14"/>
-      <c r="J50" s="14"/>
-      <c r="K50" s="14"/>
-      <c r="L50" s="14"/>
+      <c r="G50" s="13"/>
+      <c r="H50" s="13"/>
+      <c r="I50" s="13"/>
+      <c r="J50" s="13"/>
+      <c r="K50" s="13"/>
+      <c r="L50" s="13"/>
       <c r="M50" s="1"/>
     </row>
     <row r="51" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2157,24 +1954,18 @@
     </row>
     <row r="52" spans="1:13" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A52" s="1"/>
-      <c r="B52" s="13" t="s">
+      <c r="B52" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C52" s="13"/>
-      <c r="D52" s="13"/>
+      <c r="C52" s="12"/>
+      <c r="D52" s="12"/>
       <c r="E52" s="1"/>
       <c r="F52" s="1"/>
-      <c r="G52" s="15" t="str">
-        <f>_xlfn.TEXTJOIN(" / ",TRUE,_xlfn.XLOOKUP('[2]Marketing MAIL'!G7,'[2]Marketing MAIL'!K:K,'[2]Marketing MAIL'!L:L,""),_xlfn.XLOOKUP('[2]Marketing MAIL'!G8,'[2]Marketing MAIL'!K:K,'[2]Marketing MAIL'!L:L,""),_xlfn.XLOOKUP('[2]Marketing MAIL'!G9,'[2]Marketing MAIL'!K:K,'[2]Marketing MAIL'!L:L,""))</f>
-        <v>EURO STOXX 50 Index</v>
-      </c>
-      <c r="H52" s="15"/>
-      <c r="I52" s="15"/>
-      <c r="J52" s="15"/>
-      <c r="K52" s="17" t="str">
-        <f ca="1">"Startwaarde: TBD(" &amp; TEXT(WORKDAY(TODAY(),'[2]Marketing MAIL'!G25),"[$-nl-NL]d mmm yy")&amp; ")"</f>
-        <v>Startwaarde: TBD(17 apr 26)</v>
-      </c>
+      <c r="G52" s="16"/>
+      <c r="H52" s="16"/>
+      <c r="I52" s="16"/>
+      <c r="J52" s="16"/>
+      <c r="K52" s="17"/>
       <c r="L52" s="17"/>
       <c r="M52" s="1"/>
     </row>
@@ -2195,20 +1986,20 @@
     </row>
     <row r="54" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A54" s="1"/>
-      <c r="B54" s="16" t="str">
+      <c r="B54" s="14" t="str">
         <f>'[2]Marketing MAIL'!F18</f>
         <v>Premie:</v>
       </c>
-      <c r="C54" s="16"/>
-      <c r="D54" s="16"/>
+      <c r="C54" s="14"/>
+      <c r="D54" s="14"/>
       <c r="E54" s="1"/>
       <c r="F54" s="1"/>
-      <c r="G54" s="19"/>
-      <c r="H54" s="19"/>
-      <c r="I54" s="19"/>
-      <c r="J54" s="19"/>
-      <c r="K54" s="19"/>
-      <c r="L54" s="19"/>
+      <c r="G54" s="15"/>
+      <c r="H54" s="15"/>
+      <c r="I54" s="15"/>
+      <c r="J54" s="15"/>
+      <c r="K54" s="15"/>
+      <c r="L54" s="15"/>
       <c r="M54" s="1"/>
     </row>
     <row r="55" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2218,30 +2009,30 @@
       <c r="D55" s="6"/>
       <c r="E55" s="1"/>
       <c r="F55" s="1"/>
-      <c r="G55" s="21"/>
-      <c r="H55" s="21"/>
-      <c r="I55" s="21"/>
-      <c r="J55" s="21"/>
-      <c r="K55" s="21"/>
-      <c r="L55" s="21"/>
+      <c r="G55" s="7"/>
+      <c r="H55" s="7"/>
+      <c r="I55" s="7"/>
+      <c r="J55" s="7"/>
+      <c r="K55" s="7"/>
+      <c r="L55" s="7"/>
       <c r="M55" s="1"/>
     </row>
     <row r="56" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A56" s="1"/>
-      <c r="B56" s="13" t="str">
+      <c r="B56" s="12" t="str">
         <f>'[2]Marketing MAIL'!F19</f>
         <v>Aflossingsbarriere:</v>
       </c>
-      <c r="C56" s="13"/>
-      <c r="D56" s="13"/>
+      <c r="C56" s="12"/>
+      <c r="D56" s="12"/>
       <c r="E56" s="1"/>
       <c r="F56" s="1"/>
-      <c r="G56" s="19"/>
-      <c r="H56" s="19"/>
-      <c r="I56" s="19"/>
-      <c r="J56" s="19"/>
-      <c r="K56" s="19"/>
-      <c r="L56" s="19"/>
+      <c r="G56" s="15"/>
+      <c r="H56" s="15"/>
+      <c r="I56" s="15"/>
+      <c r="J56" s="15"/>
+      <c r="K56" s="15"/>
+      <c r="L56" s="15"/>
       <c r="M56" s="1"/>
     </row>
     <row r="57" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2251,30 +2042,30 @@
       <c r="D57" s="6"/>
       <c r="E57" s="1"/>
       <c r="F57" s="1"/>
-      <c r="G57" s="21"/>
-      <c r="H57" s="21"/>
-      <c r="I57" s="21"/>
-      <c r="J57" s="21"/>
-      <c r="K57" s="21"/>
-      <c r="L57" s="21"/>
+      <c r="G57" s="7"/>
+      <c r="H57" s="7"/>
+      <c r="I57" s="7"/>
+      <c r="J57" s="7"/>
+      <c r="K57" s="7"/>
+      <c r="L57" s="7"/>
       <c r="M57" s="1"/>
     </row>
     <row r="58" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A58" s="1"/>
-      <c r="B58" s="13" t="str">
+      <c r="B58" s="12" t="str">
         <f>'[2]Marketing MAIL'!F20</f>
         <v>Couponbarriere:</v>
       </c>
-      <c r="C58" s="13"/>
-      <c r="D58" s="13"/>
+      <c r="C58" s="12"/>
+      <c r="D58" s="12"/>
       <c r="E58" s="1"/>
       <c r="F58" s="1"/>
-      <c r="G58" s="19"/>
-      <c r="H58" s="19"/>
-      <c r="I58" s="19"/>
-      <c r="J58" s="19"/>
-      <c r="K58" s="19"/>
-      <c r="L58" s="19"/>
+      <c r="G58" s="15"/>
+      <c r="H58" s="15"/>
+      <c r="I58" s="15"/>
+      <c r="J58" s="15"/>
+      <c r="K58" s="15"/>
+      <c r="L58" s="15"/>
       <c r="M58" s="1"/>
     </row>
     <row r="59" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2284,30 +2075,30 @@
       <c r="D59" s="6"/>
       <c r="E59" s="1"/>
       <c r="F59" s="1"/>
-      <c r="G59" s="21"/>
-      <c r="H59" s="21"/>
-      <c r="I59" s="21"/>
-      <c r="J59" s="21"/>
-      <c r="K59" s="21"/>
-      <c r="L59" s="21"/>
+      <c r="G59" s="7"/>
+      <c r="H59" s="7"/>
+      <c r="I59" s="7"/>
+      <c r="J59" s="7"/>
+      <c r="K59" s="7"/>
+      <c r="L59" s="7"/>
       <c r="M59" s="1"/>
     </row>
     <row r="60" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A60" s="1"/>
-      <c r="B60" s="13" t="str">
+      <c r="B60" s="12" t="str">
         <f>'[2]Marketing MAIL'!F21</f>
         <v>Bescherming:</v>
       </c>
-      <c r="C60" s="13"/>
-      <c r="D60" s="13"/>
+      <c r="C60" s="12"/>
+      <c r="D60" s="12"/>
       <c r="E60" s="1"/>
       <c r="F60" s="1"/>
-      <c r="G60" s="19"/>
-      <c r="H60" s="19"/>
-      <c r="I60" s="19"/>
-      <c r="J60" s="19"/>
-      <c r="K60" s="19"/>
-      <c r="L60" s="19"/>
+      <c r="G60" s="15"/>
+      <c r="H60" s="15"/>
+      <c r="I60" s="15"/>
+      <c r="J60" s="15"/>
+      <c r="K60" s="15"/>
+      <c r="L60" s="15"/>
       <c r="M60" s="1"/>
     </row>
     <row r="61" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2371,14 +2162,7 @@
     </row>
     <row r="65" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="1"/>
-      <c r="B65" s="4" t="str">
-        <f>'[2]Marketing MAIL'!J13 &amp; " " &amp; '[2]Marketing MAIL'!J4 &amp; " " &amp;
-VLOOKUP('[2]Marketing MAIL'!J7,'[2]Marketing MAIL'!P:Q,2,FALSE)&amp;
-IF('[2]Marketing MAIL'!J9="",""," " &amp; VLOOKUP('[2]Marketing MAIL'!J9,'[2]Marketing MAIL'!P:Q,2,FALSE))&amp;
-" " &amp;
-"26-" &amp;(26+VALUE(LEFT('[2]Marketing MAIL'!J6,LEN('[2]Marketing MAIL'!J6)-1)))</f>
-        <v>VLK Memory Coupon Eurozone VS 26-33</v>
-      </c>
+      <c r="B65" s="4"/>
       <c r="C65" s="5"/>
       <c r="D65" s="5"/>
       <c r="E65" s="5"/>
@@ -2408,22 +2192,19 @@
     </row>
     <row r="67" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A67" s="1"/>
-      <c r="B67" s="13" t="s">
+      <c r="B67" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C67" s="13"/>
-      <c r="D67" s="13"/>
+      <c r="C67" s="12"/>
+      <c r="D67" s="12"/>
       <c r="E67" s="1"/>
       <c r="F67" s="1"/>
-      <c r="G67" s="14" t="str">
-        <f>_xlfn.XLOOKUP('[2]Marketing MAIL'!J13,'[2]Marketing MAIL'!F:F,'[2]Marketing MAIL'!G:G)</f>
-        <v>Van Lanschot Kempen N.V. (Fitch: A- / S&amp;P: BBB+)</v>
-      </c>
-      <c r="H67" s="14"/>
-      <c r="I67" s="14"/>
-      <c r="J67" s="14"/>
-      <c r="K67" s="14"/>
-      <c r="L67" s="14"/>
+      <c r="G67" s="13"/>
+      <c r="H67" s="13"/>
+      <c r="I67" s="13"/>
+      <c r="J67" s="13"/>
+      <c r="K67" s="13"/>
+      <c r="L67" s="13"/>
       <c r="M67" s="1"/>
     </row>
     <row r="68" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2443,22 +2224,19 @@
     </row>
     <row r="69" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A69" s="1"/>
-      <c r="B69" s="13" t="s">
+      <c r="B69" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C69" s="13"/>
-      <c r="D69" s="13"/>
+      <c r="C69" s="12"/>
+      <c r="D69" s="12"/>
       <c r="E69" s="1"/>
       <c r="F69" s="1"/>
-      <c r="G69" s="14" t="str">
-        <f ca="1">"TBD/TBD/" &amp; TEXT(WORKDAY(TODAY(),'[2]Marketing MAIL'!J5+'[2]Marketing MAIL'!J25),"d mmm yyyy")</f>
-        <v>TBD/TBD/24 Apr 2026</v>
-      </c>
-      <c r="H69" s="14"/>
-      <c r="I69" s="14"/>
-      <c r="J69" s="14"/>
-      <c r="K69" s="14"/>
-      <c r="L69" s="14"/>
+      <c r="G69" s="13"/>
+      <c r="H69" s="13"/>
+      <c r="I69" s="13"/>
+      <c r="J69" s="13"/>
+      <c r="K69" s="13"/>
+      <c r="L69" s="13"/>
       <c r="M69" s="1"/>
     </row>
     <row r="70" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2478,22 +2256,19 @@
     </row>
     <row r="71" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A71" s="1"/>
-      <c r="B71" s="13" t="s">
+      <c r="B71" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C71" s="13"/>
-      <c r="D71" s="13"/>
+      <c r="C71" s="12"/>
+      <c r="D71" s="12"/>
       <c r="E71" s="1"/>
       <c r="F71" s="1"/>
-      <c r="G71" s="14" t="str">
-        <f>'[2]Marketing MAIL'!J11 &amp; " " &amp; TEXT(_xlfn.NUMBERVALUE(SUBSTITUTE(LOWER(TRIM('[2]Marketing MAIL'!J16)),"k",""), ",", ".")*1000, "#,##0")</f>
-        <v>EUR 100,000</v>
-      </c>
-      <c r="H71" s="14"/>
-      <c r="I71" s="14"/>
-      <c r="J71" s="14"/>
-      <c r="K71" s="14"/>
-      <c r="L71" s="14"/>
+      <c r="G71" s="13"/>
+      <c r="H71" s="13"/>
+      <c r="I71" s="13"/>
+      <c r="J71" s="13"/>
+      <c r="K71" s="13"/>
+      <c r="L71" s="13"/>
       <c r="M71" s="1"/>
     </row>
     <row r="72" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2513,22 +2288,19 @@
     </row>
     <row r="73" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A73" s="1"/>
-      <c r="B73" s="13" t="s">
+      <c r="B73" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C73" s="13"/>
-      <c r="D73" s="13"/>
+      <c r="C73" s="12"/>
+      <c r="D73" s="12"/>
       <c r="E73" s="1"/>
       <c r="F73" s="1"/>
-      <c r="G73" s="14" t="str">
-        <f>SUBSTITUTE('[2]Marketing MAIL'!J6,"Y"," jaar")</f>
-        <v>7 jaar</v>
-      </c>
-      <c r="H73" s="14"/>
-      <c r="I73" s="14"/>
-      <c r="J73" s="14"/>
-      <c r="K73" s="14"/>
-      <c r="L73" s="14"/>
+      <c r="G73" s="13"/>
+      <c r="H73" s="13"/>
+      <c r="I73" s="13"/>
+      <c r="J73" s="13"/>
+      <c r="K73" s="13"/>
+      <c r="L73" s="13"/>
       <c r="M73" s="1"/>
     </row>
     <row r="74" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2548,24 +2320,18 @@
     </row>
     <row r="75" spans="1:13" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A75" s="1"/>
-      <c r="B75" s="13" t="s">
+      <c r="B75" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C75" s="13"/>
-      <c r="D75" s="13"/>
+      <c r="C75" s="12"/>
+      <c r="D75" s="12"/>
       <c r="E75" s="1"/>
       <c r="F75" s="1"/>
-      <c r="G75" s="15" t="str">
-        <f>_xlfn.TEXTJOIN(" / ",TRUE,_xlfn.XLOOKUP('[2]Marketing MAIL'!J7,'[2]Marketing MAIL'!K:K,'[2]Marketing MAIL'!L:L,""),_xlfn.XLOOKUP('[2]Marketing MAIL'!J8,'[2]Marketing MAIL'!K:K,'[2]Marketing MAIL'!L:L,""),_xlfn.XLOOKUP('[2]Marketing MAIL'!J9,'[2]Marketing MAIL'!K:K,'[2]Marketing MAIL'!L:L,""))</f>
-        <v>EURO STOXX 50 Index / S&amp;P 500</v>
-      </c>
-      <c r="H75" s="15"/>
-      <c r="I75" s="15"/>
-      <c r="J75" s="15"/>
-      <c r="K75" s="17" t="str">
-        <f ca="1">"Startwaarde: TBD(" &amp; TEXT(WORKDAY(TODAY(),'[2]Marketing MAIL'!J25),"[$-nl-NL]d mmm yy")&amp; ")"</f>
-        <v>Startwaarde: TBD(17 apr 26)</v>
-      </c>
+      <c r="G75" s="16"/>
+      <c r="H75" s="16"/>
+      <c r="I75" s="16"/>
+      <c r="J75" s="16"/>
+      <c r="K75" s="17"/>
       <c r="L75" s="17"/>
       <c r="M75" s="1"/>
     </row>
@@ -2586,20 +2352,20 @@
     </row>
     <row r="77" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A77" s="1"/>
-      <c r="B77" s="16" t="str">
+      <c r="B77" s="14" t="str">
         <f>'[2]Marketing MAIL'!I18</f>
         <v>Premie:</v>
       </c>
-      <c r="C77" s="16"/>
-      <c r="D77" s="16"/>
+      <c r="C77" s="14"/>
+      <c r="D77" s="14"/>
       <c r="E77" s="1"/>
       <c r="F77" s="1"/>
-      <c r="G77" s="19"/>
-      <c r="H77" s="19"/>
-      <c r="I77" s="19"/>
-      <c r="J77" s="19"/>
-      <c r="K77" s="19"/>
-      <c r="L77" s="19"/>
+      <c r="G77" s="15"/>
+      <c r="H77" s="15"/>
+      <c r="I77" s="15"/>
+      <c r="J77" s="15"/>
+      <c r="K77" s="15"/>
+      <c r="L77" s="15"/>
       <c r="M77" s="1"/>
     </row>
     <row r="78" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2609,30 +2375,30 @@
       <c r="D78" s="6"/>
       <c r="E78" s="1"/>
       <c r="F78" s="1"/>
-      <c r="G78" s="21"/>
-      <c r="H78" s="21"/>
-      <c r="I78" s="21"/>
-      <c r="J78" s="21"/>
-      <c r="K78" s="21"/>
-      <c r="L78" s="21"/>
+      <c r="G78" s="7"/>
+      <c r="H78" s="7"/>
+      <c r="I78" s="7"/>
+      <c r="J78" s="7"/>
+      <c r="K78" s="7"/>
+      <c r="L78" s="7"/>
       <c r="M78" s="1"/>
     </row>
     <row r="79" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A79" s="1"/>
-      <c r="B79" s="13" t="str">
+      <c r="B79" s="12" t="str">
         <f>'[2]Marketing MAIL'!I19</f>
         <v>Aflossingsbarriere:</v>
       </c>
-      <c r="C79" s="13"/>
-      <c r="D79" s="13"/>
+      <c r="C79" s="12"/>
+      <c r="D79" s="12"/>
       <c r="E79" s="1"/>
       <c r="F79" s="1"/>
-      <c r="G79" s="19"/>
-      <c r="H79" s="19"/>
-      <c r="I79" s="19"/>
-      <c r="J79" s="19"/>
-      <c r="K79" s="19"/>
-      <c r="L79" s="19"/>
+      <c r="G79" s="15"/>
+      <c r="H79" s="15"/>
+      <c r="I79" s="15"/>
+      <c r="J79" s="15"/>
+      <c r="K79" s="15"/>
+      <c r="L79" s="15"/>
       <c r="M79" s="1"/>
     </row>
     <row r="80" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2642,30 +2408,30 @@
       <c r="D80" s="6"/>
       <c r="E80" s="1"/>
       <c r="F80" s="1"/>
-      <c r="G80" s="21"/>
-      <c r="H80" s="21"/>
-      <c r="I80" s="21"/>
-      <c r="J80" s="21"/>
-      <c r="K80" s="21"/>
-      <c r="L80" s="21"/>
+      <c r="G80" s="7"/>
+      <c r="H80" s="7"/>
+      <c r="I80" s="7"/>
+      <c r="J80" s="7"/>
+      <c r="K80" s="7"/>
+      <c r="L80" s="7"/>
       <c r="M80" s="1"/>
     </row>
     <row r="81" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A81" s="1"/>
-      <c r="B81" s="13" t="str">
+      <c r="B81" s="12" t="str">
         <f>'[2]Marketing MAIL'!I20</f>
         <v>Couponbarriere:</v>
       </c>
-      <c r="C81" s="13"/>
-      <c r="D81" s="13"/>
+      <c r="C81" s="12"/>
+      <c r="D81" s="12"/>
       <c r="E81" s="1"/>
       <c r="F81" s="1"/>
-      <c r="G81" s="19"/>
-      <c r="H81" s="19"/>
-      <c r="I81" s="19"/>
-      <c r="J81" s="19"/>
-      <c r="K81" s="19"/>
-      <c r="L81" s="19"/>
+      <c r="G81" s="15"/>
+      <c r="H81" s="15"/>
+      <c r="I81" s="15"/>
+      <c r="J81" s="15"/>
+      <c r="K81" s="15"/>
+      <c r="L81" s="15"/>
       <c r="M81" s="1"/>
     </row>
     <row r="82" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2675,30 +2441,30 @@
       <c r="D82" s="6"/>
       <c r="E82" s="1"/>
       <c r="F82" s="1"/>
-      <c r="G82" s="21"/>
-      <c r="H82" s="21"/>
-      <c r="I82" s="21"/>
-      <c r="J82" s="21"/>
-      <c r="K82" s="21"/>
-      <c r="L82" s="21"/>
+      <c r="G82" s="7"/>
+      <c r="H82" s="7"/>
+      <c r="I82" s="7"/>
+      <c r="J82" s="7"/>
+      <c r="K82" s="7"/>
+      <c r="L82" s="7"/>
       <c r="M82" s="1"/>
     </row>
     <row r="83" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A83" s="1"/>
-      <c r="B83" s="13" t="str">
+      <c r="B83" s="12" t="str">
         <f>'[2]Marketing MAIL'!I21</f>
         <v>Bescherming:</v>
       </c>
-      <c r="C83" s="13"/>
-      <c r="D83" s="13"/>
+      <c r="C83" s="12"/>
+      <c r="D83" s="12"/>
       <c r="E83" s="1"/>
       <c r="F83" s="1"/>
-      <c r="G83" s="19"/>
-      <c r="H83" s="19"/>
-      <c r="I83" s="19"/>
-      <c r="J83" s="19"/>
-      <c r="K83" s="19"/>
-      <c r="L83" s="19"/>
+      <c r="G83" s="15"/>
+      <c r="H83" s="15"/>
+      <c r="I83" s="15"/>
+      <c r="J83" s="15"/>
+      <c r="K83" s="15"/>
+      <c r="L83" s="15"/>
       <c r="M83" s="1"/>
     </row>
     <row r="84" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2763,14 +2529,7 @@
     </row>
     <row r="88" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A88" s="1"/>
-      <c r="B88" s="4" t="str">
-        <f>'[2]Marketing MAIL'!M13 &amp; " " &amp; '[2]Marketing MAIL'!M4 &amp; " " &amp;
-VLOOKUP('[2]Marketing MAIL'!M7,'[2]Marketing MAIL'!P:Q,2,FALSE)&amp;
-IF('[2]Marketing MAIL'!M9="",""," " &amp; VLOOKUP('[2]Marketing MAIL'!M9,'[2]Marketing MAIL'!P:Q,2,FALSE))&amp;
-" " &amp;
-"26-" &amp;(26+VALUE(LEFT('[2]Marketing MAIL'!M6,LEN('[2]Marketing MAIL'!M6)-1)))</f>
-        <v>BNP Memory Coupon Eurozone VS 26-33</v>
-      </c>
+      <c r="B88" s="4"/>
       <c r="C88" s="5"/>
       <c r="D88" s="5"/>
       <c r="E88" s="5"/>
@@ -2800,22 +2559,19 @@
     </row>
     <row r="90" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A90" s="1"/>
-      <c r="B90" s="13" t="s">
+      <c r="B90" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C90" s="13"/>
-      <c r="D90" s="13"/>
+      <c r="C90" s="12"/>
+      <c r="D90" s="12"/>
       <c r="E90" s="1"/>
       <c r="F90" s="1"/>
-      <c r="G90" s="14" t="str">
-        <f>_xlfn.XLOOKUP('[2]Marketing MAIL'!M13,'[2]Marketing MAIL'!F:F,'[2]Marketing MAIL'!G:G)</f>
-        <v>BNP Paribas Issuance B.V. (Moody's: Aa3 / Fitch: AA- / S&amp;P: A+)</v>
-      </c>
-      <c r="H90" s="14"/>
-      <c r="I90" s="14"/>
-      <c r="J90" s="14"/>
-      <c r="K90" s="14"/>
-      <c r="L90" s="14"/>
+      <c r="G90" s="13"/>
+      <c r="H90" s="13"/>
+      <c r="I90" s="13"/>
+      <c r="J90" s="13"/>
+      <c r="K90" s="13"/>
+      <c r="L90" s="13"/>
       <c r="M90" s="1"/>
     </row>
     <row r="91" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2835,22 +2591,19 @@
     </row>
     <row r="92" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A92" s="1"/>
-      <c r="B92" s="13" t="s">
+      <c r="B92" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C92" s="13"/>
-      <c r="D92" s="13"/>
+      <c r="C92" s="12"/>
+      <c r="D92" s="12"/>
       <c r="E92" s="1"/>
       <c r="F92" s="1"/>
-      <c r="G92" s="14" t="str">
-        <f ca="1">"TBD/TBD/" &amp; TEXT(WORKDAY(TODAY(),'[2]Marketing MAIL'!M5+'[2]Marketing MAIL'!M25),"d mmm yyyy")</f>
-        <v>TBD/TBD/24 Apr 2026</v>
-      </c>
-      <c r="H92" s="14"/>
-      <c r="I92" s="14"/>
-      <c r="J92" s="14"/>
-      <c r="K92" s="14"/>
-      <c r="L92" s="14"/>
+      <c r="G92" s="13"/>
+      <c r="H92" s="13"/>
+      <c r="I92" s="13"/>
+      <c r="J92" s="13"/>
+      <c r="K92" s="13"/>
+      <c r="L92" s="13"/>
       <c r="M92" s="1"/>
     </row>
     <row r="93" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2870,22 +2623,19 @@
     </row>
     <row r="94" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A94" s="1"/>
-      <c r="B94" s="13" t="s">
+      <c r="B94" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C94" s="13"/>
-      <c r="D94" s="13"/>
+      <c r="C94" s="12"/>
+      <c r="D94" s="12"/>
       <c r="E94" s="1"/>
       <c r="F94" s="1"/>
-      <c r="G94" s="14" t="str">
-        <f>'[2]Marketing MAIL'!M11 &amp; " " &amp; TEXT(_xlfn.NUMBERVALUE(SUBSTITUTE(LOWER(TRIM('[2]Marketing MAIL'!M16)),"k",""), ",", ".")*1000, "#,##0")</f>
-        <v>EUR 100,000</v>
-      </c>
-      <c r="H94" s="14"/>
-      <c r="I94" s="14"/>
-      <c r="J94" s="14"/>
-      <c r="K94" s="14"/>
-      <c r="L94" s="14"/>
+      <c r="G94" s="13"/>
+      <c r="H94" s="13"/>
+      <c r="I94" s="13"/>
+      <c r="J94" s="13"/>
+      <c r="K94" s="13"/>
+      <c r="L94" s="13"/>
       <c r="M94" s="1"/>
     </row>
     <row r="95" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2905,22 +2655,19 @@
     </row>
     <row r="96" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A96" s="1"/>
-      <c r="B96" s="13" t="s">
+      <c r="B96" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C96" s="13"/>
-      <c r="D96" s="13"/>
+      <c r="C96" s="12"/>
+      <c r="D96" s="12"/>
       <c r="E96" s="1"/>
       <c r="F96" s="1"/>
-      <c r="G96" s="14" t="str">
-        <f>SUBSTITUTE('[2]Marketing MAIL'!M6,"Y"," jaar")</f>
-        <v>7 jaar</v>
-      </c>
-      <c r="H96" s="14"/>
-      <c r="I96" s="14"/>
-      <c r="J96" s="14"/>
-      <c r="K96" s="14"/>
-      <c r="L96" s="14"/>
+      <c r="G96" s="13"/>
+      <c r="H96" s="13"/>
+      <c r="I96" s="13"/>
+      <c r="J96" s="13"/>
+      <c r="K96" s="13"/>
+      <c r="L96" s="13"/>
       <c r="M96" s="1"/>
     </row>
     <row r="97" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2940,24 +2687,18 @@
     </row>
     <row r="98" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A98" s="1"/>
-      <c r="B98" s="13" t="s">
+      <c r="B98" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C98" s="13"/>
-      <c r="D98" s="13"/>
+      <c r="C98" s="12"/>
+      <c r="D98" s="12"/>
       <c r="E98" s="1"/>
       <c r="F98" s="1"/>
-      <c r="G98" s="15" t="str">
-        <f>_xlfn.TEXTJOIN(" / ",TRUE,_xlfn.XLOOKUP('[2]Marketing MAIL'!M7,'[2]Marketing MAIL'!K:K,'[2]Marketing MAIL'!L:L,""),_xlfn.XLOOKUP('[2]Marketing MAIL'!M8,'[2]Marketing MAIL'!K:K,'[2]Marketing MAIL'!L:L,""),_xlfn.XLOOKUP('[2]Marketing MAIL'!M9,'[2]Marketing MAIL'!K:K,'[2]Marketing MAIL'!L:L,""))</f>
-        <v>EURO STOXX 50 Index / S&amp;P 500</v>
-      </c>
-      <c r="H98" s="15"/>
-      <c r="I98" s="15"/>
-      <c r="J98" s="15"/>
-      <c r="K98" s="17" t="str">
-        <f ca="1">"Startwaarde: TBD(" &amp; TEXT(WORKDAY(TODAY(),'[2]Marketing MAIL'!J25),"[$-nl-NL]d mmm yy")&amp; ")"</f>
-        <v>Startwaarde: TBD(17 apr 26)</v>
-      </c>
+      <c r="G98" s="16"/>
+      <c r="H98" s="16"/>
+      <c r="I98" s="16"/>
+      <c r="J98" s="16"/>
+      <c r="K98" s="17"/>
       <c r="L98" s="17"/>
       <c r="M98" s="1"/>
     </row>
@@ -2978,23 +2719,20 @@
     </row>
     <row r="100" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A100" s="1"/>
-      <c r="B100" s="16" t="str">
+      <c r="B100" s="14" t="str">
         <f>'[2]Marketing MAIL'!L18</f>
         <v>Premie:</v>
       </c>
-      <c r="C100" s="16"/>
-      <c r="D100" s="16"/>
+      <c r="C100" s="14"/>
+      <c r="D100" s="14"/>
       <c r="E100" s="1"/>
       <c r="F100" s="1"/>
-      <c r="G100" s="19" t="str">
-        <f>'[2]Marketing MAIL'!M18 &amp; "%"</f>
-        <v>5.2%</v>
-      </c>
-      <c r="H100" s="19"/>
-      <c r="I100" s="19"/>
-      <c r="J100" s="19"/>
-      <c r="K100" s="19"/>
-      <c r="L100" s="19"/>
+      <c r="G100" s="15"/>
+      <c r="H100" s="15"/>
+      <c r="I100" s="15"/>
+      <c r="J100" s="15"/>
+      <c r="K100" s="15"/>
+      <c r="L100" s="15"/>
       <c r="M100" s="1"/>
     </row>
     <row r="101" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3004,33 +2742,30 @@
       <c r="D101" s="6"/>
       <c r="E101" s="1"/>
       <c r="F101" s="1"/>
-      <c r="G101" s="21"/>
-      <c r="H101" s="21"/>
-      <c r="I101" s="21"/>
-      <c r="J101" s="21"/>
-      <c r="K101" s="21"/>
-      <c r="L101" s="21"/>
+      <c r="G101" s="7"/>
+      <c r="H101" s="7"/>
+      <c r="I101" s="7"/>
+      <c r="J101" s="7"/>
+      <c r="K101" s="7"/>
+      <c r="L101" s="7"/>
       <c r="M101" s="1"/>
     </row>
     <row r="102" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A102" s="1"/>
-      <c r="B102" s="13" t="str">
+      <c r="B102" s="12" t="str">
         <f>'[2]Marketing MAIL'!L19</f>
         <v>Aflossingsbarriere:</v>
       </c>
-      <c r="C102" s="13"/>
-      <c r="D102" s="13"/>
+      <c r="C102" s="12"/>
+      <c r="D102" s="12"/>
       <c r="E102" s="1"/>
       <c r="F102" s="1"/>
-      <c r="G102" s="22" t="str">
-        <f>IF(ISBLANK('[2]Marketing MAIL'!M19),"n.v.t",'[2]Marketing MAIL'!M19 &amp; "%")</f>
-        <v>n.v.t</v>
-      </c>
-      <c r="H102" s="22"/>
-      <c r="I102" s="22"/>
-      <c r="J102" s="22"/>
-      <c r="K102" s="22"/>
-      <c r="L102" s="22"/>
+      <c r="G102" s="13"/>
+      <c r="H102" s="13"/>
+      <c r="I102" s="13"/>
+      <c r="J102" s="13"/>
+      <c r="K102" s="13"/>
+      <c r="L102" s="13"/>
       <c r="M102" s="1"/>
     </row>
     <row r="103" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3040,33 +2775,30 @@
       <c r="D103" s="6"/>
       <c r="E103" s="1"/>
       <c r="F103" s="1"/>
-      <c r="G103" s="21"/>
-      <c r="H103" s="21"/>
-      <c r="I103" s="21"/>
-      <c r="J103" s="21"/>
-      <c r="K103" s="21"/>
-      <c r="L103" s="21"/>
+      <c r="G103" s="7"/>
+      <c r="H103" s="7"/>
+      <c r="I103" s="7"/>
+      <c r="J103" s="7"/>
+      <c r="K103" s="7"/>
+      <c r="L103" s="7"/>
       <c r="M103" s="1"/>
     </row>
     <row r="104" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A104" s="1"/>
-      <c r="B104" s="13" t="str">
+      <c r="B104" s="12" t="str">
         <f>'[2]Marketing MAIL'!L20</f>
         <v>Couponbarriere:</v>
       </c>
-      <c r="C104" s="13"/>
-      <c r="D104" s="13"/>
+      <c r="C104" s="12"/>
+      <c r="D104" s="12"/>
       <c r="E104" s="1"/>
       <c r="F104" s="1"/>
-      <c r="G104" s="22" t="str">
-        <f>IF(ISBLANK('[2]Marketing MAIL'!M20),"n.v.t",'[2]Marketing MAIL'!M20 &amp; "%")</f>
-        <v>n.v.t</v>
-      </c>
-      <c r="H104" s="22"/>
-      <c r="I104" s="22"/>
-      <c r="J104" s="22"/>
-      <c r="K104" s="22"/>
-      <c r="L104" s="22"/>
+      <c r="G104" s="13"/>
+      <c r="H104" s="13"/>
+      <c r="I104" s="13"/>
+      <c r="J104" s="13"/>
+      <c r="K104" s="13"/>
+      <c r="L104" s="13"/>
       <c r="M104" s="1"/>
     </row>
     <row r="105" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3076,33 +2808,30 @@
       <c r="D105" s="6"/>
       <c r="E105" s="1"/>
       <c r="F105" s="1"/>
-      <c r="G105" s="21"/>
-      <c r="H105" s="21"/>
-      <c r="I105" s="21"/>
-      <c r="J105" s="21"/>
-      <c r="K105" s="21"/>
-      <c r="L105" s="21"/>
+      <c r="G105" s="7"/>
+      <c r="H105" s="7"/>
+      <c r="I105" s="7"/>
+      <c r="J105" s="7"/>
+      <c r="K105" s="7"/>
+      <c r="L105" s="7"/>
       <c r="M105" s="1"/>
     </row>
     <row r="106" spans="1:13" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A106" s="1"/>
-      <c r="B106" s="13" t="str">
+      <c r="B106" s="12" t="str">
         <f>'[2]Marketing MAIL'!L21</f>
         <v>Bescherming:</v>
       </c>
-      <c r="C106" s="13"/>
-      <c r="D106" s="13"/>
+      <c r="C106" s="12"/>
+      <c r="D106" s="12"/>
       <c r="E106" s="1"/>
       <c r="F106" s="1"/>
-      <c r="G106" s="22" t="str">
-        <f>IF(ISBLANK('[2]Marketing MAIL'!M21),"n.v.t",'[2]Marketing MAIL'!M21 &amp; "%")</f>
-        <v>n.v.t</v>
-      </c>
-      <c r="H106" s="22"/>
-      <c r="I106" s="22"/>
-      <c r="J106" s="22"/>
-      <c r="K106" s="22"/>
-      <c r="L106" s="22"/>
+      <c r="G106" s="13"/>
+      <c r="H106" s="13"/>
+      <c r="I106" s="13"/>
+      <c r="J106" s="13"/>
+      <c r="K106" s="13"/>
+      <c r="L106" s="13"/>
       <c r="M106" s="1"/>
     </row>
     <row r="107" spans="1:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3142,50 +2871,28 @@
     </row>
   </sheetData>
   <mergeCells count="82">
-    <mergeCell ref="B102:D102"/>
-    <mergeCell ref="G102:L102"/>
-    <mergeCell ref="B104:D104"/>
-    <mergeCell ref="G104:L104"/>
-    <mergeCell ref="B106:D106"/>
-    <mergeCell ref="G106:L106"/>
-    <mergeCell ref="B100:D100"/>
-    <mergeCell ref="G100:L100"/>
-    <mergeCell ref="B90:D90"/>
-    <mergeCell ref="G90:L90"/>
-    <mergeCell ref="B92:D92"/>
-    <mergeCell ref="G92:L92"/>
-    <mergeCell ref="B94:D94"/>
-    <mergeCell ref="G94:L94"/>
-    <mergeCell ref="B96:D96"/>
-    <mergeCell ref="G96:L96"/>
-    <mergeCell ref="B98:D98"/>
-    <mergeCell ref="G98:J98"/>
-    <mergeCell ref="K98:L98"/>
-    <mergeCell ref="B79:D79"/>
-    <mergeCell ref="G79:L79"/>
-    <mergeCell ref="B81:D81"/>
-    <mergeCell ref="G81:L81"/>
-    <mergeCell ref="B83:D83"/>
-    <mergeCell ref="G83:L83"/>
-    <mergeCell ref="B77:D77"/>
-    <mergeCell ref="G77:L77"/>
-    <mergeCell ref="B67:D67"/>
-    <mergeCell ref="G67:L67"/>
-    <mergeCell ref="B69:D69"/>
-    <mergeCell ref="G69:L69"/>
-    <mergeCell ref="B71:D71"/>
-    <mergeCell ref="G71:L71"/>
-    <mergeCell ref="B73:D73"/>
-    <mergeCell ref="G73:L73"/>
-    <mergeCell ref="B75:D75"/>
-    <mergeCell ref="G75:J75"/>
-    <mergeCell ref="K75:L75"/>
-    <mergeCell ref="B56:D56"/>
-    <mergeCell ref="G56:L56"/>
-    <mergeCell ref="B58:D58"/>
-    <mergeCell ref="G58:L58"/>
-    <mergeCell ref="B60:D60"/>
-    <mergeCell ref="G60:L60"/>
+    <mergeCell ref="R10:W10"/>
+    <mergeCell ref="B12:L17"/>
+    <mergeCell ref="R12:W12"/>
+    <mergeCell ref="R14:W14"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="G22:L22"/>
+    <mergeCell ref="R30:U30"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="G32:L32"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="G24:L24"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="G26:L26"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="G28:L28"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="G38:L38"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="G30:J30"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="G34:L34"/>
     <mergeCell ref="R34:S34"/>
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="G36:L36"/>
@@ -3202,28 +2909,50 @@
     <mergeCell ref="B52:D52"/>
     <mergeCell ref="G52:J52"/>
     <mergeCell ref="K52:L52"/>
-    <mergeCell ref="B38:D38"/>
-    <mergeCell ref="G38:L38"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="G30:J30"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="G34:L34"/>
-    <mergeCell ref="R30:U30"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="G32:L32"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="G24:L24"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="G26:L26"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="G28:L28"/>
-    <mergeCell ref="R10:W10"/>
-    <mergeCell ref="B12:L17"/>
-    <mergeCell ref="R12:W12"/>
-    <mergeCell ref="R14:W14"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="G22:L22"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="G56:L56"/>
+    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="G58:L58"/>
+    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="G60:L60"/>
+    <mergeCell ref="B77:D77"/>
+    <mergeCell ref="G77:L77"/>
+    <mergeCell ref="B67:D67"/>
+    <mergeCell ref="G67:L67"/>
+    <mergeCell ref="B69:D69"/>
+    <mergeCell ref="G69:L69"/>
+    <mergeCell ref="B71:D71"/>
+    <mergeCell ref="G71:L71"/>
+    <mergeCell ref="B73:D73"/>
+    <mergeCell ref="G73:L73"/>
+    <mergeCell ref="B75:D75"/>
+    <mergeCell ref="G75:J75"/>
+    <mergeCell ref="K75:L75"/>
+    <mergeCell ref="B79:D79"/>
+    <mergeCell ref="G79:L79"/>
+    <mergeCell ref="B81:D81"/>
+    <mergeCell ref="G81:L81"/>
+    <mergeCell ref="B83:D83"/>
+    <mergeCell ref="G83:L83"/>
+    <mergeCell ref="B100:D100"/>
+    <mergeCell ref="G100:L100"/>
+    <mergeCell ref="B90:D90"/>
+    <mergeCell ref="G90:L90"/>
+    <mergeCell ref="B92:D92"/>
+    <mergeCell ref="G92:L92"/>
+    <mergeCell ref="B94:D94"/>
+    <mergeCell ref="G94:L94"/>
+    <mergeCell ref="B96:D96"/>
+    <mergeCell ref="G96:L96"/>
+    <mergeCell ref="B98:D98"/>
+    <mergeCell ref="G98:J98"/>
+    <mergeCell ref="K98:L98"/>
+    <mergeCell ref="B102:D102"/>
+    <mergeCell ref="G102:L102"/>
+    <mergeCell ref="B104:D104"/>
+    <mergeCell ref="G104:L104"/>
+    <mergeCell ref="B106:D106"/>
+    <mergeCell ref="G106:L106"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>